<commit_message>
Atualização automática: 2026-09-21 08:59
</commit_message>
<xml_diff>
--- a/dados/base/bpo.xlsx
+++ b/dados/base/bpo.xlsx
@@ -1879,7 +1879,7 @@
         <v>46283</v>
       </c>
       <c r="M10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N10" t="s">
         <v>221</v>
@@ -1947,7 +1947,7 @@
         <v>46283</v>
       </c>
       <c r="M11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N11" t="s">
         <v>221</v>
@@ -2015,7 +2015,7 @@
         <v>46283</v>
       </c>
       <c r="M12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N12" t="s">
         <v>221</v>
@@ -4123,7 +4123,7 @@
         <v>46283</v>
       </c>
       <c r="M43" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N43" t="s">
         <v>221</v>
@@ -4191,7 +4191,7 @@
         <v>46283</v>
       </c>
       <c r="M44" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N44" t="s">
         <v>221</v>
@@ -4259,7 +4259,7 @@
         <v>46283</v>
       </c>
       <c r="M45" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N45" t="s">
         <v>221</v>
@@ -5687,7 +5687,7 @@
         <v>46283</v>
       </c>
       <c r="M66" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N66" t="s">
         <v>221</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-30 10:13
</commit_message>
<xml_diff>
--- a/dados/base/bpo.xlsx
+++ b/dados/base/bpo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12224" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12227" uniqueCount="288">
   <si>
     <t>CodCliente</t>
   </si>
@@ -493,10 +493,10 @@
     <t>B.P.O. - DELTA</t>
   </si>
   <si>
-    <t>B.P.O. - GUARANI</t>
+    <t>ROSSI - CTB</t>
   </si>
   <si>
-    <t>ROSSI - CTB</t>
+    <t>B.P.O. - GUARANI</t>
   </si>
   <si>
     <t>B.P.O. - GUARANI EF</t>
@@ -5006,31 +5006,31 @@
     </row>
     <row r="56" spans="1:33">
       <c r="A56">
-        <v>4064</v>
+        <v>2371</v>
       </c>
       <c r="B56" t="s">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="C56" t="s">
         <v>141</v>
       </c>
       <c r="D56" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E56" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F56" t="s">
         <v>147</v>
       </c>
       <c r="G56">
-        <v>9312</v>
+        <v>3790</v>
       </c>
       <c r="H56">
         <v>0</v>
       </c>
       <c r="I56" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="J56" t="s">
         <v>175</v>
@@ -5045,10 +5045,10 @@
         <v>220</v>
       </c>
       <c r="O56">
-        <v>17841025</v>
+        <v>17540512</v>
       </c>
       <c r="P56" t="s">
-        <v>224</v>
+        <v>147</v>
       </c>
       <c r="Q56" t="s">
         <v>236</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="T56" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="U56" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="W56" t="s">
         <v>254</v>
@@ -5074,16 +5074,16 @@
     </row>
     <row r="57" spans="1:33">
       <c r="A57">
-        <v>4917</v>
+        <v>3366</v>
       </c>
       <c r="B57" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C57" t="s">
         <v>141</v>
       </c>
       <c r="D57" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E57" t="s">
         <v>147</v>
@@ -5092,13 +5092,13 @@
         <v>147</v>
       </c>
       <c r="G57">
-        <v>9312</v>
+        <v>3790</v>
       </c>
       <c r="H57">
         <v>0</v>
       </c>
       <c r="I57" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="J57" t="s">
         <v>175</v>
@@ -5113,10 +5113,10 @@
         <v>220</v>
       </c>
       <c r="O57">
-        <v>17629841</v>
+        <v>17448656</v>
       </c>
       <c r="P57" t="s">
-        <v>224</v>
+        <v>147</v>
       </c>
       <c r="Q57" t="s">
         <v>236</v>
@@ -5125,10 +5125,10 @@
         <v>0</v>
       </c>
       <c r="T57" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="U57" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="W57" t="s">
         <v>254</v>
@@ -5142,16 +5142,16 @@
     </row>
     <row r="58" spans="1:33">
       <c r="A58">
-        <v>4917</v>
+        <v>2371</v>
       </c>
       <c r="B58" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C58" t="s">
         <v>141</v>
       </c>
       <c r="D58" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E58" t="s">
         <v>147</v>
@@ -5160,13 +5160,13 @@
         <v>147</v>
       </c>
       <c r="G58">
-        <v>9277</v>
+        <v>2152</v>
       </c>
       <c r="H58">
         <v>0</v>
       </c>
       <c r="I58" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="J58" t="s">
         <v>176</v>
@@ -5181,10 +5181,10 @@
         <v>220</v>
       </c>
       <c r="O58">
-        <v>17629821</v>
+        <v>17540411</v>
       </c>
       <c r="P58" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="Q58" t="s">
         <v>236</v>
@@ -5193,13 +5193,13 @@
         <v>0</v>
       </c>
       <c r="T58" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="U58" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="W58" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AA58">
         <v>0</v>
@@ -5210,16 +5210,16 @@
     </row>
     <row r="59" spans="1:33">
       <c r="A59">
-        <v>2371</v>
+        <v>3366</v>
       </c>
       <c r="B59" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C59" t="s">
         <v>141</v>
       </c>
       <c r="D59" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E59" t="s">
         <v>147</v>
@@ -5228,16 +5228,16 @@
         <v>147</v>
       </c>
       <c r="G59">
-        <v>3790</v>
+        <v>2152</v>
       </c>
       <c r="H59">
         <v>0</v>
       </c>
       <c r="I59" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="J59" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="L59" s="1">
         <v>46295</v>
@@ -5249,10 +5249,10 @@
         <v>220</v>
       </c>
       <c r="O59">
-        <v>17540512</v>
+        <v>17448596</v>
       </c>
       <c r="P59" t="s">
-        <v>147</v>
+        <v>228</v>
       </c>
       <c r="Q59" t="s">
         <v>236</v>
@@ -5267,7 +5267,7 @@
         <v>244</v>
       </c>
       <c r="W59" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="AA59">
         <v>0</v>
@@ -5278,146 +5278,152 @@
     </row>
     <row r="60" spans="1:33">
       <c r="A60">
-        <v>3366</v>
+        <v>2804</v>
       </c>
       <c r="B60" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="C60" t="s">
         <v>141</v>
       </c>
       <c r="D60" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E60" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F60" t="s">
         <v>147</v>
       </c>
       <c r="G60">
-        <v>3790</v>
+        <v>7040</v>
       </c>
       <c r="H60">
         <v>0</v>
       </c>
       <c r="I60" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="J60" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="L60" s="1">
-        <v>46295</v>
-      </c>
-      <c r="M60" t="s">
-        <v>211</v>
+        <v>46280</v>
       </c>
       <c r="N60" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O60">
-        <v>17448656</v>
+        <v>17326612</v>
       </c>
       <c r="P60" t="s">
-        <v>147</v>
+        <v>227</v>
       </c>
       <c r="Q60" t="s">
-        <v>236</v>
+        <v>237</v>
+      </c>
+      <c r="R60" s="1">
+        <v>46280.72560332176</v>
       </c>
       <c r="S60">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T60" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="U60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="W60" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="AA60">
         <v>0</v>
       </c>
+      <c r="AB60" t="s">
+        <v>279</v>
+      </c>
       <c r="AG60" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="61" spans="1:33">
       <c r="A61">
-        <v>2371</v>
+        <v>2835</v>
       </c>
       <c r="B61" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="C61" t="s">
         <v>141</v>
       </c>
       <c r="D61" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E61" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F61" t="s">
         <v>147</v>
       </c>
       <c r="G61">
-        <v>2152</v>
+        <v>7040</v>
       </c>
       <c r="H61">
         <v>0</v>
       </c>
       <c r="I61" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="J61" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="L61" s="1">
-        <v>46295</v>
-      </c>
-      <c r="M61" t="s">
-        <v>211</v>
+        <v>46280</v>
       </c>
       <c r="N61" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O61">
-        <v>17540411</v>
+        <v>17089972</v>
       </c>
       <c r="P61" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="Q61" t="s">
-        <v>236</v>
+        <v>237</v>
+      </c>
+      <c r="R61" s="1">
+        <v>46282.47436697916</v>
       </c>
       <c r="S61">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T61" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="U61" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="W61" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AA61">
         <v>0</v>
       </c>
+      <c r="AB61" t="s">
+        <v>279</v>
+      </c>
       <c r="AG61" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="62" spans="1:33">
       <c r="A62">
-        <v>3366</v>
+        <v>2837</v>
       </c>
       <c r="B62" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="C62" t="s">
         <v>141</v>
@@ -5426,72 +5432,75 @@
         <v>142</v>
       </c>
       <c r="E62" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F62" t="s">
         <v>147</v>
       </c>
       <c r="G62">
-        <v>2152</v>
+        <v>7040</v>
       </c>
       <c r="H62">
         <v>0</v>
       </c>
       <c r="I62" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="J62" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="L62" s="1">
-        <v>46295</v>
-      </c>
-      <c r="M62" t="s">
-        <v>211</v>
+        <v>46280</v>
       </c>
       <c r="N62" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O62">
-        <v>17448596</v>
+        <v>17582284</v>
       </c>
       <c r="P62" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="Q62" t="s">
-        <v>236</v>
+        <v>237</v>
+      </c>
+      <c r="R62" s="1">
+        <v>46282.4745590625</v>
       </c>
       <c r="S62">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="T62" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="U62" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="W62" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AA62">
         <v>0</v>
       </c>
+      <c r="AB62" t="s">
+        <v>279</v>
+      </c>
       <c r="AG62" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="63" spans="1:33">
       <c r="A63">
-        <v>2804</v>
+        <v>2838</v>
       </c>
       <c r="B63" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C63" t="s">
         <v>141</v>
       </c>
       <c r="D63" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E63" t="s">
         <v>148</v>
@@ -5518,7 +5527,7 @@
         <v>221</v>
       </c>
       <c r="O63">
-        <v>17326612</v>
+        <v>17389995</v>
       </c>
       <c r="P63" t="s">
         <v>227</v>
@@ -5527,7 +5536,7 @@
         <v>237</v>
       </c>
       <c r="R63" s="1">
-        <v>46280.72560332176</v>
+        <v>46282.4739224537</v>
       </c>
       <c r="S63">
         <v>15</v>
@@ -5553,19 +5562,19 @@
     </row>
     <row r="64" spans="1:33">
       <c r="A64">
-        <v>2835</v>
+        <v>2842</v>
       </c>
       <c r="B64" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C64" t="s">
         <v>141</v>
       </c>
       <c r="D64" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E64" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F64" t="s">
         <v>147</v>
@@ -5589,7 +5598,7 @@
         <v>221</v>
       </c>
       <c r="O64">
-        <v>17089972</v>
+        <v>17161658</v>
       </c>
       <c r="P64" t="s">
         <v>227</v>
@@ -5598,7 +5607,7 @@
         <v>237</v>
       </c>
       <c r="R64" s="1">
-        <v>46282.47436697916</v>
+        <v>46282.47498869213</v>
       </c>
       <c r="S64">
         <v>15</v>
@@ -5624,10 +5633,10 @@
     </row>
     <row r="65" spans="1:33">
       <c r="A65">
-        <v>2837</v>
+        <v>3004</v>
       </c>
       <c r="B65" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C65" t="s">
         <v>141</v>
@@ -5660,7 +5669,7 @@
         <v>221</v>
       </c>
       <c r="O65">
-        <v>17582284</v>
+        <v>17033285</v>
       </c>
       <c r="P65" t="s">
         <v>227</v>
@@ -5669,7 +5678,7 @@
         <v>237</v>
       </c>
       <c r="R65" s="1">
-        <v>46282.4745590625</v>
+        <v>46282.47512175926</v>
       </c>
       <c r="S65">
         <v>15</v>
@@ -5695,10 +5704,10 @@
     </row>
     <row r="66" spans="1:33">
       <c r="A66">
-        <v>2838</v>
+        <v>3005</v>
       </c>
       <c r="B66" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C66" t="s">
         <v>141</v>
@@ -5731,7 +5740,7 @@
         <v>221</v>
       </c>
       <c r="O66">
-        <v>17389995</v>
+        <v>17263482</v>
       </c>
       <c r="P66" t="s">
         <v>227</v>
@@ -5740,7 +5749,7 @@
         <v>237</v>
       </c>
       <c r="R66" s="1">
-        <v>46282.4739224537</v>
+        <v>46282.47529371528</v>
       </c>
       <c r="S66">
         <v>15</v>
@@ -5766,19 +5775,19 @@
     </row>
     <row r="67" spans="1:33">
       <c r="A67">
-        <v>2842</v>
+        <v>3039</v>
       </c>
       <c r="B67" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C67" t="s">
         <v>141</v>
       </c>
       <c r="D67" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E67" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F67" t="s">
         <v>147</v>
@@ -5802,7 +5811,7 @@
         <v>221</v>
       </c>
       <c r="O67">
-        <v>17161658</v>
+        <v>17585738</v>
       </c>
       <c r="P67" t="s">
         <v>227</v>
@@ -5811,7 +5820,7 @@
         <v>237</v>
       </c>
       <c r="R67" s="1">
-        <v>46282.47498869213</v>
+        <v>46282.47544363426</v>
       </c>
       <c r="S67">
         <v>15</v>
@@ -5837,16 +5846,16 @@
     </row>
     <row r="68" spans="1:33">
       <c r="A68">
-        <v>3004</v>
+        <v>3053</v>
       </c>
       <c r="B68" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C68" t="s">
         <v>141</v>
       </c>
       <c r="D68" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E68" t="s">
         <v>148</v>
@@ -5873,7 +5882,7 @@
         <v>221</v>
       </c>
       <c r="O68">
-        <v>17033285</v>
+        <v>17194136</v>
       </c>
       <c r="P68" t="s">
         <v>227</v>
@@ -5882,7 +5891,7 @@
         <v>237</v>
       </c>
       <c r="R68" s="1">
-        <v>46282.47512175926</v>
+        <v>46282.47562407408</v>
       </c>
       <c r="S68">
         <v>15</v>
@@ -5908,10 +5917,10 @@
     </row>
     <row r="69" spans="1:33">
       <c r="A69">
-        <v>3005</v>
+        <v>3209</v>
       </c>
       <c r="B69" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C69" t="s">
         <v>141</v>
@@ -5920,7 +5929,7 @@
         <v>142</v>
       </c>
       <c r="E69" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F69" t="s">
         <v>147</v>
@@ -5944,7 +5953,7 @@
         <v>221</v>
       </c>
       <c r="O69">
-        <v>17263482</v>
+        <v>17135070</v>
       </c>
       <c r="P69" t="s">
         <v>227</v>
@@ -5953,7 +5962,7 @@
         <v>237</v>
       </c>
       <c r="R69" s="1">
-        <v>46282.47529371528</v>
+        <v>46282.4758247338</v>
       </c>
       <c r="S69">
         <v>15</v>
@@ -5979,10 +5988,10 @@
     </row>
     <row r="70" spans="1:33">
       <c r="A70">
-        <v>3039</v>
+        <v>3480</v>
       </c>
       <c r="B70" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C70" t="s">
         <v>141</v>
@@ -6015,7 +6024,7 @@
         <v>221</v>
       </c>
       <c r="O70">
-        <v>17585738</v>
+        <v>17821480</v>
       </c>
       <c r="P70" t="s">
         <v>227</v>
@@ -6024,7 +6033,7 @@
         <v>237</v>
       </c>
       <c r="R70" s="1">
-        <v>46282.47544363426</v>
+        <v>46282.47608140046</v>
       </c>
       <c r="S70">
         <v>15</v>
@@ -6050,16 +6059,16 @@
     </row>
     <row r="71" spans="1:33">
       <c r="A71">
-        <v>3053</v>
+        <v>3481</v>
       </c>
       <c r="B71" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C71" t="s">
         <v>141</v>
       </c>
       <c r="D71" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E71" t="s">
         <v>148</v>
@@ -6086,7 +6095,7 @@
         <v>221</v>
       </c>
       <c r="O71">
-        <v>17194136</v>
+        <v>17333186</v>
       </c>
       <c r="P71" t="s">
         <v>227</v>
@@ -6095,7 +6104,7 @@
         <v>237</v>
       </c>
       <c r="R71" s="1">
-        <v>46282.47562407408</v>
+        <v>46282.47626608796</v>
       </c>
       <c r="S71">
         <v>15</v>
@@ -6121,25 +6130,25 @@
     </row>
     <row r="72" spans="1:33">
       <c r="A72">
-        <v>3209</v>
+        <v>2804</v>
       </c>
       <c r="B72" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="C72" t="s">
         <v>141</v>
       </c>
       <c r="D72" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E72" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F72" t="s">
         <v>147</v>
       </c>
       <c r="G72">
-        <v>7040</v>
+        <v>7041</v>
       </c>
       <c r="H72">
         <v>0</v>
@@ -6148,16 +6157,16 @@
         <v>158</v>
       </c>
       <c r="J72" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="L72" s="1">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="N72" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O72">
-        <v>17135070</v>
+        <v>17326621</v>
       </c>
       <c r="P72" t="s">
         <v>227</v>
@@ -6166,10 +6175,10 @@
         <v>237</v>
       </c>
       <c r="R72" s="1">
-        <v>46282.4758247338</v>
+        <v>46268.39249731482</v>
       </c>
       <c r="S72">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="T72" t="s">
         <v>241</v>
@@ -6177,14 +6186,11 @@
       <c r="U72" t="s">
         <v>243</v>
       </c>
-      <c r="W72" t="s">
-        <v>256</v>
-      </c>
       <c r="AA72">
         <v>0</v>
       </c>
       <c r="AB72" t="s">
-        <v>279</v>
+        <v>227</v>
       </c>
       <c r="AG72" t="s">
         <v>285</v>
@@ -6192,10 +6198,10 @@
     </row>
     <row r="73" spans="1:33">
       <c r="A73">
-        <v>3480</v>
+        <v>2835</v>
       </c>
       <c r="B73" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C73" t="s">
         <v>141</v>
@@ -6210,7 +6216,7 @@
         <v>147</v>
       </c>
       <c r="G73">
-        <v>7040</v>
+        <v>7041</v>
       </c>
       <c r="H73">
         <v>0</v>
@@ -6219,16 +6225,16 @@
         <v>158</v>
       </c>
       <c r="J73" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="L73" s="1">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="N73" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O73">
-        <v>17821480</v>
+        <v>17089997</v>
       </c>
       <c r="P73" t="s">
         <v>227</v>
@@ -6237,10 +6243,10 @@
         <v>237</v>
       </c>
       <c r="R73" s="1">
-        <v>46282.47608140046</v>
+        <v>46268.39249833333</v>
       </c>
       <c r="S73">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="T73" t="s">
         <v>241</v>
@@ -6248,14 +6254,11 @@
       <c r="U73" t="s">
         <v>243</v>
       </c>
-      <c r="W73" t="s">
-        <v>256</v>
-      </c>
       <c r="AA73">
         <v>0</v>
       </c>
       <c r="AB73" t="s">
-        <v>279</v>
+        <v>227</v>
       </c>
       <c r="AG73" t="s">
         <v>285</v>
@@ -6263,10 +6266,10 @@
     </row>
     <row r="74" spans="1:33">
       <c r="A74">
-        <v>3481</v>
+        <v>2837</v>
       </c>
       <c r="B74" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C74" t="s">
         <v>141</v>
@@ -6281,7 +6284,7 @@
         <v>147</v>
       </c>
       <c r="G74">
-        <v>7040</v>
+        <v>7041</v>
       </c>
       <c r="H74">
         <v>0</v>
@@ -6290,16 +6293,16 @@
         <v>158</v>
       </c>
       <c r="J74" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="L74" s="1">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="N74" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O74">
-        <v>17333186</v>
+        <v>17582293</v>
       </c>
       <c r="P74" t="s">
         <v>227</v>
@@ -6308,10 +6311,10 @@
         <v>237</v>
       </c>
       <c r="R74" s="1">
-        <v>46282.47626608796</v>
+        <v>46268.39249914352</v>
       </c>
       <c r="S74">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="T74" t="s">
         <v>241</v>
@@ -6319,14 +6322,11 @@
       <c r="U74" t="s">
         <v>243</v>
       </c>
-      <c r="W74" t="s">
-        <v>256</v>
-      </c>
       <c r="AA74">
         <v>0</v>
       </c>
       <c r="AB74" t="s">
-        <v>279</v>
+        <v>227</v>
       </c>
       <c r="AG74" t="s">
         <v>285</v>
@@ -6334,16 +6334,16 @@
     </row>
     <row r="75" spans="1:33">
       <c r="A75">
-        <v>2804</v>
+        <v>2838</v>
       </c>
       <c r="B75" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C75" t="s">
         <v>141</v>
       </c>
       <c r="D75" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E75" t="s">
         <v>148</v>
@@ -6370,7 +6370,7 @@
         <v>220</v>
       </c>
       <c r="O75">
-        <v>17326621</v>
+        <v>17390004</v>
       </c>
       <c r="P75" t="s">
         <v>227</v>
@@ -6379,7 +6379,7 @@
         <v>237</v>
       </c>
       <c r="R75" s="1">
-        <v>46268.39249731482</v>
+        <v>46268.39250015046</v>
       </c>
       <c r="S75">
         <v>29</v>
@@ -6402,19 +6402,19 @@
     </row>
     <row r="76" spans="1:33">
       <c r="A76">
-        <v>2835</v>
+        <v>2842</v>
       </c>
       <c r="B76" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C76" t="s">
         <v>141</v>
       </c>
       <c r="D76" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E76" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F76" t="s">
         <v>147</v>
@@ -6438,7 +6438,7 @@
         <v>220</v>
       </c>
       <c r="O76">
-        <v>17089997</v>
+        <v>17161680</v>
       </c>
       <c r="P76" t="s">
         <v>227</v>
@@ -6447,7 +6447,7 @@
         <v>237</v>
       </c>
       <c r="R76" s="1">
-        <v>46268.39249833333</v>
+        <v>46268.39250150463</v>
       </c>
       <c r="S76">
         <v>29</v>
@@ -6470,10 +6470,10 @@
     </row>
     <row r="77" spans="1:33">
       <c r="A77">
-        <v>2837</v>
+        <v>3004</v>
       </c>
       <c r="B77" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C77" t="s">
         <v>141</v>
@@ -6506,7 +6506,7 @@
         <v>220</v>
       </c>
       <c r="O77">
-        <v>17582293</v>
+        <v>17033305</v>
       </c>
       <c r="P77" t="s">
         <v>227</v>
@@ -6515,7 +6515,7 @@
         <v>237</v>
       </c>
       <c r="R77" s="1">
-        <v>46268.39249914352</v>
+        <v>46268.39250226852</v>
       </c>
       <c r="S77">
         <v>29</v>
@@ -6538,10 +6538,10 @@
     </row>
     <row r="78" spans="1:33">
       <c r="A78">
-        <v>2838</v>
+        <v>3005</v>
       </c>
       <c r="B78" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C78" t="s">
         <v>141</v>
@@ -6574,7 +6574,7 @@
         <v>220</v>
       </c>
       <c r="O78">
-        <v>17390004</v>
+        <v>17263491</v>
       </c>
       <c r="P78" t="s">
         <v>227</v>
@@ -6583,7 +6583,7 @@
         <v>237</v>
       </c>
       <c r="R78" s="1">
-        <v>46268.39250015046</v>
+        <v>46268.39250332176</v>
       </c>
       <c r="S78">
         <v>29</v>
@@ -6606,19 +6606,19 @@
     </row>
     <row r="79" spans="1:33">
       <c r="A79">
-        <v>2842</v>
+        <v>3039</v>
       </c>
       <c r="B79" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C79" t="s">
         <v>141</v>
       </c>
       <c r="D79" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E79" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F79" t="s">
         <v>147</v>
@@ -6642,7 +6642,7 @@
         <v>220</v>
       </c>
       <c r="O79">
-        <v>17161680</v>
+        <v>17585747</v>
       </c>
       <c r="P79" t="s">
         <v>227</v>
@@ -6651,7 +6651,7 @@
         <v>237</v>
       </c>
       <c r="R79" s="1">
-        <v>46268.39250150463</v>
+        <v>46268.39250452547</v>
       </c>
       <c r="S79">
         <v>29</v>
@@ -6674,16 +6674,16 @@
     </row>
     <row r="80" spans="1:33">
       <c r="A80">
-        <v>3004</v>
+        <v>3053</v>
       </c>
       <c r="B80" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C80" t="s">
         <v>141</v>
       </c>
       <c r="D80" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E80" t="s">
         <v>148</v>
@@ -6710,7 +6710,7 @@
         <v>220</v>
       </c>
       <c r="O80">
-        <v>17033305</v>
+        <v>17194164</v>
       </c>
       <c r="P80" t="s">
         <v>227</v>
@@ -6719,7 +6719,7 @@
         <v>237</v>
       </c>
       <c r="R80" s="1">
-        <v>46268.39250226852</v>
+        <v>46268.39250524306</v>
       </c>
       <c r="S80">
         <v>29</v>
@@ -6742,10 +6742,10 @@
     </row>
     <row r="81" spans="1:33">
       <c r="A81">
-        <v>3005</v>
+        <v>3209</v>
       </c>
       <c r="B81" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C81" t="s">
         <v>141</v>
@@ -6754,7 +6754,7 @@
         <v>142</v>
       </c>
       <c r="E81" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F81" t="s">
         <v>147</v>
@@ -6778,7 +6778,7 @@
         <v>220</v>
       </c>
       <c r="O81">
-        <v>17263491</v>
+        <v>17135091</v>
       </c>
       <c r="P81" t="s">
         <v>227</v>
@@ -6787,7 +6787,7 @@
         <v>237</v>
       </c>
       <c r="R81" s="1">
-        <v>46268.39250332176</v>
+        <v>46268.39250652778</v>
       </c>
       <c r="S81">
         <v>29</v>
@@ -6810,10 +6810,10 @@
     </row>
     <row r="82" spans="1:33">
       <c r="A82">
-        <v>3039</v>
+        <v>3480</v>
       </c>
       <c r="B82" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C82" t="s">
         <v>141</v>
@@ -6846,7 +6846,7 @@
         <v>220</v>
       </c>
       <c r="O82">
-        <v>17585747</v>
+        <v>17821489</v>
       </c>
       <c r="P82" t="s">
         <v>227</v>
@@ -6855,7 +6855,7 @@
         <v>237</v>
       </c>
       <c r="R82" s="1">
-        <v>46268.39250452547</v>
+        <v>46268.39250747685</v>
       </c>
       <c r="S82">
         <v>29</v>
@@ -6878,16 +6878,16 @@
     </row>
     <row r="83" spans="1:33">
       <c r="A83">
-        <v>3053</v>
+        <v>3481</v>
       </c>
       <c r="B83" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C83" t="s">
         <v>141</v>
       </c>
       <c r="D83" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E83" t="s">
         <v>148</v>
@@ -6914,7 +6914,7 @@
         <v>220</v>
       </c>
       <c r="O83">
-        <v>17194164</v>
+        <v>17333195</v>
       </c>
       <c r="P83" t="s">
         <v>227</v>
@@ -6923,7 +6923,7 @@
         <v>237</v>
       </c>
       <c r="R83" s="1">
-        <v>46268.39250524306</v>
+        <v>46268.39250818287</v>
       </c>
       <c r="S83">
         <v>29</v>
@@ -6946,25 +6946,25 @@
     </row>
     <row r="84" spans="1:33">
       <c r="A84">
-        <v>3209</v>
+        <v>2804</v>
       </c>
       <c r="B84" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="C84" t="s">
         <v>141</v>
       </c>
       <c r="D84" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E84" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F84" t="s">
         <v>147</v>
       </c>
       <c r="G84">
-        <v>7041</v>
+        <v>11289</v>
       </c>
       <c r="H84">
         <v>0</v>
@@ -6973,16 +6973,16 @@
         <v>158</v>
       </c>
       <c r="J84" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="L84" s="1">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="N84" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O84">
-        <v>17135091</v>
+        <v>17326643</v>
       </c>
       <c r="P84" t="s">
         <v>227</v>
@@ -6991,10 +6991,10 @@
         <v>237</v>
       </c>
       <c r="R84" s="1">
-        <v>46268.39250652778</v>
+        <v>46280.7143515162</v>
       </c>
       <c r="S84">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="T84" t="s">
         <v>241</v>
@@ -7014,16 +7014,16 @@
     </row>
     <row r="85" spans="1:33">
       <c r="A85">
-        <v>3480</v>
+        <v>3053</v>
       </c>
       <c r="B85" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C85" t="s">
         <v>141</v>
       </c>
       <c r="D85" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E85" t="s">
         <v>148</v>
@@ -7032,7 +7032,7 @@
         <v>147</v>
       </c>
       <c r="G85">
-        <v>7041</v>
+        <v>11289</v>
       </c>
       <c r="H85">
         <v>0</v>
@@ -7041,16 +7041,16 @@
         <v>158</v>
       </c>
       <c r="J85" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="L85" s="1">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="N85" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O85">
-        <v>17821489</v>
+        <v>17194213</v>
       </c>
       <c r="P85" t="s">
         <v>227</v>
@@ -7059,10 +7059,10 @@
         <v>237</v>
       </c>
       <c r="R85" s="1">
-        <v>46268.39250747685</v>
+        <v>46280.71435333334</v>
       </c>
       <c r="S85">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="T85" t="s">
         <v>241</v>
@@ -7082,16 +7082,16 @@
     </row>
     <row r="86" spans="1:33">
       <c r="A86">
-        <v>3481</v>
+        <v>2804</v>
       </c>
       <c r="B86" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C86" t="s">
         <v>141</v>
       </c>
       <c r="D86" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E86" t="s">
         <v>148</v>
@@ -7100,7 +7100,7 @@
         <v>147</v>
       </c>
       <c r="G86">
-        <v>7041</v>
+        <v>11288</v>
       </c>
       <c r="H86">
         <v>0</v>
@@ -7109,16 +7109,16 @@
         <v>158</v>
       </c>
       <c r="J86" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L86" s="1">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N86" t="s">
         <v>220</v>
       </c>
       <c r="O86">
-        <v>17333195</v>
+        <v>17326632</v>
       </c>
       <c r="P86" t="s">
         <v>227</v>
@@ -7127,10 +7127,10 @@
         <v>237</v>
       </c>
       <c r="R86" s="1">
-        <v>46268.39250818287</v>
+        <v>46268.39323719907</v>
       </c>
       <c r="S86">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T86" t="s">
         <v>241</v>
@@ -7150,16 +7150,16 @@
     </row>
     <row r="87" spans="1:33">
       <c r="A87">
-        <v>2804</v>
+        <v>3053</v>
       </c>
       <c r="B87" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C87" t="s">
         <v>141</v>
       </c>
       <c r="D87" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E87" t="s">
         <v>148</v>
@@ -7168,7 +7168,7 @@
         <v>147</v>
       </c>
       <c r="G87">
-        <v>11289</v>
+        <v>11288</v>
       </c>
       <c r="H87">
         <v>0</v>
@@ -7177,16 +7177,16 @@
         <v>158</v>
       </c>
       <c r="J87" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="L87" s="1">
-        <v>46281</v>
+        <v>46267</v>
       </c>
       <c r="N87" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O87">
-        <v>17326643</v>
+        <v>17194186</v>
       </c>
       <c r="P87" t="s">
         <v>227</v>
@@ -7195,10 +7195,10 @@
         <v>237</v>
       </c>
       <c r="R87" s="1">
-        <v>46280.7143515162</v>
+        <v>46268.39323780093</v>
       </c>
       <c r="S87">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="T87" t="s">
         <v>241</v>
@@ -7218,10 +7218,10 @@
     </row>
     <row r="88" spans="1:33">
       <c r="A88">
-        <v>3053</v>
+        <v>4064</v>
       </c>
       <c r="B88" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="C88" t="s">
         <v>141</v>
@@ -7230,182 +7230,194 @@
         <v>143</v>
       </c>
       <c r="E88" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F88" t="s">
         <v>147</v>
       </c>
       <c r="G88">
-        <v>11289</v>
+        <v>9312</v>
       </c>
       <c r="H88">
         <v>0</v>
       </c>
       <c r="I88" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J88" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="L88" s="1">
-        <v>46281</v>
+        <v>46295</v>
+      </c>
+      <c r="M88" t="s">
+        <v>211</v>
       </c>
       <c r="N88" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O88">
-        <v>17194213</v>
+        <v>17841025</v>
       </c>
       <c r="P88" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="Q88" t="s">
         <v>237</v>
       </c>
       <c r="R88" s="1">
-        <v>46280.71435333334</v>
+        <v>46295.40172307871</v>
       </c>
       <c r="S88">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="T88" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="U88" t="s">
         <v>243</v>
       </c>
+      <c r="W88" t="s">
+        <v>254</v>
+      </c>
       <c r="AA88">
         <v>0</v>
       </c>
       <c r="AB88" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AG88" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="89" spans="1:33">
       <c r="A89">
-        <v>2804</v>
+        <v>4917</v>
       </c>
       <c r="B89" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="C89" t="s">
         <v>141</v>
       </c>
       <c r="D89" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E89" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F89" t="s">
         <v>147</v>
       </c>
       <c r="G89">
-        <v>11288</v>
+        <v>9312</v>
       </c>
       <c r="H89">
         <v>0</v>
       </c>
       <c r="I89" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J89" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L89" s="1">
-        <v>46267</v>
+        <v>46295</v>
+      </c>
+      <c r="M89" t="s">
+        <v>211</v>
       </c>
       <c r="N89" t="s">
         <v>220</v>
       </c>
       <c r="O89">
-        <v>17326632</v>
+        <v>17629841</v>
       </c>
       <c r="P89" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="Q89" t="s">
         <v>237</v>
       </c>
       <c r="R89" s="1">
-        <v>46268.39323719907</v>
+        <v>46295.40172364583</v>
       </c>
       <c r="S89">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="T89" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="U89" t="s">
         <v>243</v>
       </c>
+      <c r="W89" t="s">
+        <v>254</v>
+      </c>
       <c r="AA89">
         <v>0</v>
       </c>
       <c r="AB89" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AG89" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="90" spans="1:33">
       <c r="A90">
-        <v>3053</v>
+        <v>4059</v>
       </c>
       <c r="B90" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C90" t="s">
         <v>141</v>
       </c>
       <c r="D90" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E90" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F90" t="s">
         <v>147</v>
       </c>
       <c r="G90">
-        <v>11288</v>
+        <v>9327</v>
       </c>
       <c r="H90">
         <v>0</v>
       </c>
       <c r="I90" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J90" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="L90" s="1">
-        <v>46267</v>
+        <v>46280</v>
       </c>
       <c r="N90" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O90">
-        <v>17194186</v>
+        <v>17311887</v>
       </c>
       <c r="P90" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="Q90" t="s">
         <v>237</v>
       </c>
       <c r="R90" s="1">
-        <v>46268.39323780093</v>
+        <v>46280.75157195602</v>
       </c>
       <c r="S90">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="T90" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="U90" t="s">
         <v>243</v>
@@ -7414,27 +7426,27 @@
         <v>0</v>
       </c>
       <c r="AB90" t="s">
-        <v>227</v>
+        <v>279</v>
       </c>
       <c r="AG90" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="91" spans="1:33">
       <c r="A91">
-        <v>4059</v>
+        <v>4064</v>
       </c>
       <c r="B91" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C91" t="s">
         <v>141</v>
       </c>
       <c r="D91" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E91" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F91" t="s">
         <v>147</v>
@@ -7446,7 +7458,7 @@
         <v>0</v>
       </c>
       <c r="I91" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J91" t="s">
         <v>168</v>
@@ -7458,7 +7470,7 @@
         <v>221</v>
       </c>
       <c r="O91">
-        <v>17311887</v>
+        <v>17841036</v>
       </c>
       <c r="P91" t="s">
         <v>224</v>
@@ -7467,7 +7479,7 @@
         <v>237</v>
       </c>
       <c r="R91" s="1">
-        <v>46280.75157195602</v>
+        <v>46280.75190127315</v>
       </c>
       <c r="S91">
         <v>15</v>
@@ -7490,19 +7502,19 @@
     </row>
     <row r="92" spans="1:33">
       <c r="A92">
-        <v>4064</v>
+        <v>4065</v>
       </c>
       <c r="B92" t="s">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="C92" t="s">
         <v>141</v>
       </c>
       <c r="D92" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E92" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F92" t="s">
         <v>147</v>
@@ -7514,7 +7526,7 @@
         <v>0</v>
       </c>
       <c r="I92" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J92" t="s">
         <v>168</v>
@@ -7526,7 +7538,7 @@
         <v>221</v>
       </c>
       <c r="O92">
-        <v>17841036</v>
+        <v>17222004</v>
       </c>
       <c r="P92" t="s">
         <v>224</v>
@@ -7535,7 +7547,7 @@
         <v>237</v>
       </c>
       <c r="R92" s="1">
-        <v>46280.75190127315</v>
+        <v>46280.75219267361</v>
       </c>
       <c r="S92">
         <v>15</v>
@@ -7558,10 +7570,10 @@
     </row>
     <row r="93" spans="1:33">
       <c r="A93">
-        <v>4065</v>
+        <v>4066</v>
       </c>
       <c r="B93" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C93" t="s">
         <v>141</v>
@@ -7570,7 +7582,7 @@
         <v>142</v>
       </c>
       <c r="E93" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F93" t="s">
         <v>147</v>
@@ -7582,7 +7594,7 @@
         <v>0</v>
       </c>
       <c r="I93" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J93" t="s">
         <v>168</v>
@@ -7594,7 +7606,7 @@
         <v>221</v>
       </c>
       <c r="O93">
-        <v>17222004</v>
+        <v>17424451</v>
       </c>
       <c r="P93" t="s">
         <v>224</v>
@@ -7603,7 +7615,7 @@
         <v>237</v>
       </c>
       <c r="R93" s="1">
-        <v>46280.75219267361</v>
+        <v>46280.75248533565</v>
       </c>
       <c r="S93">
         <v>15</v>
@@ -7626,10 +7638,10 @@
     </row>
     <row r="94" spans="1:33">
       <c r="A94">
-        <v>4066</v>
+        <v>4067</v>
       </c>
       <c r="B94" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C94" t="s">
         <v>141</v>
@@ -7638,7 +7650,7 @@
         <v>142</v>
       </c>
       <c r="E94" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F94" t="s">
         <v>147</v>
@@ -7650,7 +7662,7 @@
         <v>0</v>
       </c>
       <c r="I94" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J94" t="s">
         <v>168</v>
@@ -7662,7 +7674,7 @@
         <v>221</v>
       </c>
       <c r="O94">
-        <v>17424451</v>
+        <v>17493444</v>
       </c>
       <c r="P94" t="s">
         <v>224</v>
@@ -7671,7 +7683,7 @@
         <v>237</v>
       </c>
       <c r="R94" s="1">
-        <v>46280.75248533565</v>
+        <v>46280.75296913194</v>
       </c>
       <c r="S94">
         <v>15</v>
@@ -7694,10 +7706,10 @@
     </row>
     <row r="95" spans="1:33">
       <c r="A95">
-        <v>4067</v>
+        <v>4068</v>
       </c>
       <c r="B95" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C95" t="s">
         <v>141</v>
@@ -7718,7 +7730,7 @@
         <v>0</v>
       </c>
       <c r="I95" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J95" t="s">
         <v>168</v>
@@ -7730,7 +7742,7 @@
         <v>221</v>
       </c>
       <c r="O95">
-        <v>17493444</v>
+        <v>17424491</v>
       </c>
       <c r="P95" t="s">
         <v>224</v>
@@ -7739,7 +7751,7 @@
         <v>237</v>
       </c>
       <c r="R95" s="1">
-        <v>46280.75296913194</v>
+        <v>46280.75326030092</v>
       </c>
       <c r="S95">
         <v>15</v>
@@ -7762,10 +7774,10 @@
     </row>
     <row r="96" spans="1:33">
       <c r="A96">
-        <v>4068</v>
+        <v>4602</v>
       </c>
       <c r="B96" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C96" t="s">
         <v>141</v>
@@ -7786,7 +7798,7 @@
         <v>0</v>
       </c>
       <c r="I96" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J96" t="s">
         <v>168</v>
@@ -7798,7 +7810,7 @@
         <v>221</v>
       </c>
       <c r="O96">
-        <v>17424491</v>
+        <v>17719860</v>
       </c>
       <c r="P96" t="s">
         <v>224</v>
@@ -7807,7 +7819,7 @@
         <v>237</v>
       </c>
       <c r="R96" s="1">
-        <v>46280.75326030092</v>
+        <v>46280.75372538195</v>
       </c>
       <c r="S96">
         <v>15</v>
@@ -7830,10 +7842,10 @@
     </row>
     <row r="97" spans="1:33">
       <c r="A97">
-        <v>4602</v>
+        <v>4815</v>
       </c>
       <c r="B97" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="C97" t="s">
         <v>141</v>
@@ -7854,7 +7866,7 @@
         <v>0</v>
       </c>
       <c r="I97" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J97" t="s">
         <v>168</v>
@@ -7866,7 +7878,7 @@
         <v>221</v>
       </c>
       <c r="O97">
-        <v>17719860</v>
+        <v>17728390</v>
       </c>
       <c r="P97" t="s">
         <v>224</v>
@@ -7875,7 +7887,7 @@
         <v>237</v>
       </c>
       <c r="R97" s="1">
-        <v>46280.75372538195</v>
+        <v>46280.75461721064</v>
       </c>
       <c r="S97">
         <v>15</v>
@@ -7898,16 +7910,16 @@
     </row>
     <row r="98" spans="1:33">
       <c r="A98">
-        <v>4815</v>
+        <v>4917</v>
       </c>
       <c r="B98" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C98" t="s">
         <v>141</v>
       </c>
       <c r="D98" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E98" t="s">
         <v>147</v>
@@ -7922,7 +7934,7 @@
         <v>0</v>
       </c>
       <c r="I98" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J98" t="s">
         <v>168</v>
@@ -7934,7 +7946,7 @@
         <v>221</v>
       </c>
       <c r="O98">
-        <v>17728390</v>
+        <v>17629852</v>
       </c>
       <c r="P98" t="s">
         <v>224</v>
@@ -7943,7 +7955,7 @@
         <v>237</v>
       </c>
       <c r="R98" s="1">
-        <v>46280.75461721064</v>
+        <v>46280.75492121528</v>
       </c>
       <c r="S98">
         <v>15</v>
@@ -7966,16 +7978,16 @@
     </row>
     <row r="99" spans="1:33">
       <c r="A99">
-        <v>4917</v>
+        <v>4059</v>
       </c>
       <c r="B99" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="C99" t="s">
         <v>141</v>
       </c>
       <c r="D99" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E99" t="s">
         <v>147</v>
@@ -7984,25 +7996,25 @@
         <v>147</v>
       </c>
       <c r="G99">
-        <v>9327</v>
+        <v>9328</v>
       </c>
       <c r="H99">
         <v>0</v>
       </c>
       <c r="I99" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J99" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="L99" s="1">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="N99" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O99">
-        <v>17629852</v>
+        <v>17311896</v>
       </c>
       <c r="P99" t="s">
         <v>224</v>
@@ -8011,10 +8023,10 @@
         <v>237</v>
       </c>
       <c r="R99" s="1">
-        <v>46280.75492121528</v>
+        <v>46266.71710929398</v>
       </c>
       <c r="S99">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="T99" t="s">
         <v>238</v>
@@ -8034,19 +8046,19 @@
     </row>
     <row r="100" spans="1:33">
       <c r="A100">
-        <v>4059</v>
+        <v>4064</v>
       </c>
       <c r="B100" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C100" t="s">
         <v>141</v>
       </c>
       <c r="D100" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E100" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F100" t="s">
         <v>147</v>
@@ -8058,7 +8070,7 @@
         <v>0</v>
       </c>
       <c r="I100" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J100" t="s">
         <v>177</v>
@@ -8070,7 +8082,7 @@
         <v>220</v>
       </c>
       <c r="O100">
-        <v>17311896</v>
+        <v>17841045</v>
       </c>
       <c r="P100" t="s">
         <v>224</v>
@@ -8079,7 +8091,7 @@
         <v>237</v>
       </c>
       <c r="R100" s="1">
-        <v>46266.71710929398</v>
+        <v>46266.71760243056</v>
       </c>
       <c r="S100">
         <v>29</v>
@@ -8102,19 +8114,19 @@
     </row>
     <row r="101" spans="1:33">
       <c r="A101">
-        <v>4064</v>
+        <v>4065</v>
       </c>
       <c r="B101" t="s">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="C101" t="s">
         <v>141</v>
       </c>
       <c r="D101" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E101" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F101" t="s">
         <v>147</v>
@@ -8126,7 +8138,7 @@
         <v>0</v>
       </c>
       <c r="I101" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J101" t="s">
         <v>177</v>
@@ -8138,7 +8150,7 @@
         <v>220</v>
       </c>
       <c r="O101">
-        <v>17841045</v>
+        <v>17222030</v>
       </c>
       <c r="P101" t="s">
         <v>224</v>
@@ -8147,7 +8159,7 @@
         <v>237</v>
       </c>
       <c r="R101" s="1">
-        <v>46266.71760243056</v>
+        <v>46266.71793020833</v>
       </c>
       <c r="S101">
         <v>29</v>
@@ -8170,10 +8182,10 @@
     </row>
     <row r="102" spans="1:33">
       <c r="A102">
-        <v>4065</v>
+        <v>4066</v>
       </c>
       <c r="B102" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C102" t="s">
         <v>141</v>
@@ -8182,7 +8194,7 @@
         <v>142</v>
       </c>
       <c r="E102" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F102" t="s">
         <v>147</v>
@@ -8194,7 +8206,7 @@
         <v>0</v>
       </c>
       <c r="I102" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J102" t="s">
         <v>177</v>
@@ -8206,7 +8218,7 @@
         <v>220</v>
       </c>
       <c r="O102">
-        <v>17222030</v>
+        <v>17424460</v>
       </c>
       <c r="P102" t="s">
         <v>224</v>
@@ -8215,7 +8227,7 @@
         <v>237</v>
       </c>
       <c r="R102" s="1">
-        <v>46266.71793020833</v>
+        <v>46266.71818136574</v>
       </c>
       <c r="S102">
         <v>29</v>
@@ -8238,10 +8250,10 @@
     </row>
     <row r="103" spans="1:33">
       <c r="A103">
-        <v>4066</v>
+        <v>4067</v>
       </c>
       <c r="B103" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C103" t="s">
         <v>141</v>
@@ -8250,7 +8262,7 @@
         <v>142</v>
       </c>
       <c r="E103" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F103" t="s">
         <v>147</v>
@@ -8262,7 +8274,7 @@
         <v>0</v>
       </c>
       <c r="I103" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J103" t="s">
         <v>177</v>
@@ -8274,7 +8286,7 @@
         <v>220</v>
       </c>
       <c r="O103">
-        <v>17424460</v>
+        <v>17493453</v>
       </c>
       <c r="P103" t="s">
         <v>224</v>
@@ -8283,7 +8295,7 @@
         <v>237</v>
       </c>
       <c r="R103" s="1">
-        <v>46266.71818136574</v>
+        <v>46266.71859741898</v>
       </c>
       <c r="S103">
         <v>29</v>
@@ -8306,10 +8318,10 @@
     </row>
     <row r="104" spans="1:33">
       <c r="A104">
-        <v>4067</v>
+        <v>4068</v>
       </c>
       <c r="B104" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C104" t="s">
         <v>141</v>
@@ -8330,7 +8342,7 @@
         <v>0</v>
       </c>
       <c r="I104" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J104" t="s">
         <v>177</v>
@@ -8342,7 +8354,7 @@
         <v>220</v>
       </c>
       <c r="O104">
-        <v>17493453</v>
+        <v>17424500</v>
       </c>
       <c r="P104" t="s">
         <v>224</v>
@@ -8351,7 +8363,7 @@
         <v>237</v>
       </c>
       <c r="R104" s="1">
-        <v>46266.71859741898</v>
+        <v>46266.71905170139</v>
       </c>
       <c r="S104">
         <v>29</v>
@@ -8374,10 +8386,10 @@
     </row>
     <row r="105" spans="1:33">
       <c r="A105">
-        <v>4068</v>
+        <v>4602</v>
       </c>
       <c r="B105" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C105" t="s">
         <v>141</v>
@@ -8398,7 +8410,7 @@
         <v>0</v>
       </c>
       <c r="I105" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J105" t="s">
         <v>177</v>
@@ -8410,7 +8422,7 @@
         <v>220</v>
       </c>
       <c r="O105">
-        <v>17424500</v>
+        <v>17719869</v>
       </c>
       <c r="P105" t="s">
         <v>224</v>
@@ -8419,7 +8431,7 @@
         <v>237</v>
       </c>
       <c r="R105" s="1">
-        <v>46266.71905170139</v>
+        <v>46266.71958452546</v>
       </c>
       <c r="S105">
         <v>29</v>
@@ -8442,10 +8454,10 @@
     </row>
     <row r="106" spans="1:33">
       <c r="A106">
-        <v>4602</v>
+        <v>4815</v>
       </c>
       <c r="B106" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="C106" t="s">
         <v>141</v>
@@ -8466,7 +8478,7 @@
         <v>0</v>
       </c>
       <c r="I106" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J106" t="s">
         <v>177</v>
@@ -8478,7 +8490,7 @@
         <v>220</v>
       </c>
       <c r="O106">
-        <v>17719869</v>
+        <v>17728399</v>
       </c>
       <c r="P106" t="s">
         <v>224</v>
@@ -8487,7 +8499,7 @@
         <v>237</v>
       </c>
       <c r="R106" s="1">
-        <v>46266.71958452546</v>
+        <v>46266.71982650463</v>
       </c>
       <c r="S106">
         <v>29</v>
@@ -8510,16 +8522,16 @@
     </row>
     <row r="107" spans="1:33">
       <c r="A107">
-        <v>4815</v>
+        <v>4917</v>
       </c>
       <c r="B107" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C107" t="s">
         <v>141</v>
       </c>
       <c r="D107" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E107" t="s">
         <v>147</v>
@@ -8534,7 +8546,7 @@
         <v>0</v>
       </c>
       <c r="I107" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J107" t="s">
         <v>177</v>
@@ -8546,7 +8558,7 @@
         <v>220</v>
       </c>
       <c r="O107">
-        <v>17728399</v>
+        <v>17629861</v>
       </c>
       <c r="P107" t="s">
         <v>224</v>
@@ -8555,7 +8567,7 @@
         <v>237</v>
       </c>
       <c r="R107" s="1">
-        <v>46266.71982650463</v>
+        <v>46266.72010234954</v>
       </c>
       <c r="S107">
         <v>29</v>
@@ -8578,16 +8590,16 @@
     </row>
     <row r="108" spans="1:33">
       <c r="A108">
-        <v>4917</v>
+        <v>4059</v>
       </c>
       <c r="B108" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="C108" t="s">
         <v>141</v>
       </c>
       <c r="D108" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E108" t="s">
         <v>147</v>
@@ -8596,25 +8608,25 @@
         <v>147</v>
       </c>
       <c r="G108">
-        <v>9328</v>
+        <v>9588</v>
       </c>
       <c r="H108">
         <v>0</v>
       </c>
       <c r="I108" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J108" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="L108" s="1">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="N108" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O108">
-        <v>17629861</v>
+        <v>17311917</v>
       </c>
       <c r="P108" t="s">
         <v>224</v>
@@ -8623,10 +8635,10 @@
         <v>237</v>
       </c>
       <c r="R108" s="1">
-        <v>46266.72010234954</v>
+        <v>46281.61917107639</v>
       </c>
       <c r="S108">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="T108" t="s">
         <v>238</v>
@@ -8638,10 +8650,10 @@
         <v>0</v>
       </c>
       <c r="AB108" t="s">
-        <v>279</v>
+        <v>224</v>
       </c>
       <c r="AG108" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="109" spans="1:33">
@@ -8664,13 +8676,13 @@
         <v>147</v>
       </c>
       <c r="G109">
-        <v>9588</v>
+        <v>9600</v>
       </c>
       <c r="H109">
         <v>0</v>
       </c>
       <c r="I109" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J109" t="s">
         <v>169</v>
@@ -8678,11 +8690,14 @@
       <c r="L109" s="1">
         <v>46281</v>
       </c>
+      <c r="M109" t="s">
+        <v>212</v>
+      </c>
       <c r="N109" t="s">
         <v>221</v>
       </c>
       <c r="O109">
-        <v>17311917</v>
+        <v>17311927</v>
       </c>
       <c r="P109" t="s">
         <v>224</v>
@@ -8691,7 +8706,7 @@
         <v>237</v>
       </c>
       <c r="R109" s="1">
-        <v>46281.61917107639</v>
+        <v>46286.74416417824</v>
       </c>
       <c r="S109">
         <v>14</v>
@@ -8702,6 +8717,9 @@
       <c r="U109" t="s">
         <v>243</v>
       </c>
+      <c r="W109" t="s">
+        <v>257</v>
+      </c>
       <c r="AA109">
         <v>0</v>
       </c>
@@ -8714,10 +8732,10 @@
     </row>
     <row r="110" spans="1:33">
       <c r="A110">
-        <v>4059</v>
+        <v>4061</v>
       </c>
       <c r="B110" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C110" t="s">
         <v>141</v>
@@ -8726,19 +8744,19 @@
         <v>144</v>
       </c>
       <c r="E110" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F110" t="s">
         <v>147</v>
       </c>
       <c r="G110">
-        <v>9600</v>
+        <v>9588</v>
       </c>
       <c r="H110">
         <v>0</v>
       </c>
       <c r="I110" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J110" t="s">
         <v>169</v>
@@ -8746,14 +8764,11 @@
       <c r="L110" s="1">
         <v>46281</v>
       </c>
-      <c r="M110" t="s">
-        <v>212</v>
-      </c>
       <c r="N110" t="s">
         <v>221</v>
       </c>
       <c r="O110">
-        <v>17311927</v>
+        <v>17311967</v>
       </c>
       <c r="P110" t="s">
         <v>224</v>
@@ -8762,7 +8777,7 @@
         <v>237</v>
       </c>
       <c r="R110" s="1">
-        <v>46286.74416417824</v>
+        <v>46281.61917159722</v>
       </c>
       <c r="S110">
         <v>14</v>
@@ -8772,9 +8787,6 @@
       </c>
       <c r="U110" t="s">
         <v>243</v>
-      </c>
-      <c r="W110" t="s">
-        <v>257</v>
       </c>
       <c r="AA110">
         <v>0</v>
@@ -8806,13 +8818,13 @@
         <v>147</v>
       </c>
       <c r="G111">
-        <v>9588</v>
+        <v>9600</v>
       </c>
       <c r="H111">
         <v>0</v>
       </c>
       <c r="I111" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J111" t="s">
         <v>169</v>
@@ -8820,11 +8832,14 @@
       <c r="L111" s="1">
         <v>46281</v>
       </c>
+      <c r="M111" t="s">
+        <v>212</v>
+      </c>
       <c r="N111" t="s">
         <v>221</v>
       </c>
       <c r="O111">
-        <v>17311967</v>
+        <v>17311977</v>
       </c>
       <c r="P111" t="s">
         <v>224</v>
@@ -8833,7 +8848,7 @@
         <v>237</v>
       </c>
       <c r="R111" s="1">
-        <v>46281.61917159722</v>
+        <v>46286.74416459491</v>
       </c>
       <c r="S111">
         <v>14</v>
@@ -8844,6 +8859,9 @@
       <c r="U111" t="s">
         <v>243</v>
       </c>
+      <c r="W111" t="s">
+        <v>258</v>
+      </c>
       <c r="AA111">
         <v>0</v>
       </c>
@@ -8856,10 +8874,10 @@
     </row>
     <row r="112" spans="1:33">
       <c r="A112">
-        <v>4061</v>
+        <v>4062</v>
       </c>
       <c r="B112" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C112" t="s">
         <v>141</v>
@@ -8868,19 +8886,19 @@
         <v>144</v>
       </c>
       <c r="E112" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F112" t="s">
         <v>147</v>
       </c>
       <c r="G112">
-        <v>9600</v>
+        <v>9588</v>
       </c>
       <c r="H112">
         <v>0</v>
       </c>
       <c r="I112" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J112" t="s">
         <v>169</v>
@@ -8888,14 +8906,11 @@
       <c r="L112" s="1">
         <v>46281</v>
       </c>
-      <c r="M112" t="s">
-        <v>212</v>
-      </c>
       <c r="N112" t="s">
         <v>221</v>
       </c>
       <c r="O112">
-        <v>17311977</v>
+        <v>17756707</v>
       </c>
       <c r="P112" t="s">
         <v>224</v>
@@ -8904,7 +8919,7 @@
         <v>237</v>
       </c>
       <c r="R112" s="1">
-        <v>46286.74416459491</v>
+        <v>46281.61917203703</v>
       </c>
       <c r="S112">
         <v>14</v>
@@ -8914,9 +8929,6 @@
       </c>
       <c r="U112" t="s">
         <v>243</v>
-      </c>
-      <c r="W112" t="s">
-        <v>258</v>
       </c>
       <c r="AA112">
         <v>0</v>
@@ -8948,13 +8960,13 @@
         <v>147</v>
       </c>
       <c r="G113">
-        <v>9588</v>
+        <v>9600</v>
       </c>
       <c r="H113">
         <v>0</v>
       </c>
       <c r="I113" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J113" t="s">
         <v>169</v>
@@ -8962,11 +8974,14 @@
       <c r="L113" s="1">
         <v>46281</v>
       </c>
+      <c r="M113" t="s">
+        <v>212</v>
+      </c>
       <c r="N113" t="s">
         <v>221</v>
       </c>
       <c r="O113">
-        <v>17756707</v>
+        <v>17756717</v>
       </c>
       <c r="P113" t="s">
         <v>224</v>
@@ -8975,7 +8990,7 @@
         <v>237</v>
       </c>
       <c r="R113" s="1">
-        <v>46281.61917203703</v>
+        <v>46286.74416505787</v>
       </c>
       <c r="S113">
         <v>14</v>
@@ -8986,6 +9001,9 @@
       <c r="U113" t="s">
         <v>243</v>
       </c>
+      <c r="W113" t="s">
+        <v>258</v>
+      </c>
       <c r="AA113">
         <v>0</v>
       </c>
@@ -8998,10 +9016,10 @@
     </row>
     <row r="114" spans="1:33">
       <c r="A114">
-        <v>4062</v>
+        <v>4063</v>
       </c>
       <c r="B114" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C114" t="s">
         <v>141</v>
@@ -9010,19 +9028,19 @@
         <v>144</v>
       </c>
       <c r="E114" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F114" t="s">
         <v>147</v>
       </c>
       <c r="G114">
-        <v>9600</v>
+        <v>9588</v>
       </c>
       <c r="H114">
         <v>0</v>
       </c>
       <c r="I114" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J114" t="s">
         <v>169</v>
@@ -9030,14 +9048,11 @@
       <c r="L114" s="1">
         <v>46281</v>
       </c>
-      <c r="M114" t="s">
-        <v>212</v>
-      </c>
       <c r="N114" t="s">
         <v>221</v>
       </c>
       <c r="O114">
-        <v>17756717</v>
+        <v>17221886</v>
       </c>
       <c r="P114" t="s">
         <v>224</v>
@@ -9046,7 +9061,7 @@
         <v>237</v>
       </c>
       <c r="R114" s="1">
-        <v>46286.74416505787</v>
+        <v>46281.6191725</v>
       </c>
       <c r="S114">
         <v>14</v>
@@ -9056,9 +9071,6 @@
       </c>
       <c r="U114" t="s">
         <v>243</v>
-      </c>
-      <c r="W114" t="s">
-        <v>258</v>
       </c>
       <c r="AA114">
         <v>0</v>
@@ -9090,13 +9102,13 @@
         <v>147</v>
       </c>
       <c r="G115">
-        <v>9588</v>
+        <v>9600</v>
       </c>
       <c r="H115">
         <v>0</v>
       </c>
       <c r="I115" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J115" t="s">
         <v>169</v>
@@ -9104,11 +9116,14 @@
       <c r="L115" s="1">
         <v>46281</v>
       </c>
+      <c r="M115" t="s">
+        <v>212</v>
+      </c>
       <c r="N115" t="s">
         <v>221</v>
       </c>
       <c r="O115">
-        <v>17221886</v>
+        <v>17221914</v>
       </c>
       <c r="P115" t="s">
         <v>224</v>
@@ -9117,7 +9132,7 @@
         <v>237</v>
       </c>
       <c r="R115" s="1">
-        <v>46281.6191725</v>
+        <v>46286.74416604167</v>
       </c>
       <c r="S115">
         <v>14</v>
@@ -9128,6 +9143,9 @@
       <c r="U115" t="s">
         <v>243</v>
       </c>
+      <c r="W115" t="s">
+        <v>258</v>
+      </c>
       <c r="AA115">
         <v>0</v>
       </c>
@@ -9140,10 +9158,10 @@
     </row>
     <row r="116" spans="1:33">
       <c r="A116">
-        <v>4063</v>
+        <v>4535</v>
       </c>
       <c r="B116" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C116" t="s">
         <v>141</v>
@@ -9152,19 +9170,19 @@
         <v>144</v>
       </c>
       <c r="E116" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F116" t="s">
         <v>147</v>
       </c>
       <c r="G116">
-        <v>9600</v>
+        <v>9588</v>
       </c>
       <c r="H116">
         <v>0</v>
       </c>
       <c r="I116" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J116" t="s">
         <v>169</v>
@@ -9172,14 +9190,11 @@
       <c r="L116" s="1">
         <v>46281</v>
       </c>
-      <c r="M116" t="s">
-        <v>212</v>
-      </c>
       <c r="N116" t="s">
         <v>221</v>
       </c>
       <c r="O116">
-        <v>17221914</v>
+        <v>17260697</v>
       </c>
       <c r="P116" t="s">
         <v>224</v>
@@ -9188,7 +9203,7 @@
         <v>237</v>
       </c>
       <c r="R116" s="1">
-        <v>46286.74416604167</v>
+        <v>46281.61917288195</v>
       </c>
       <c r="S116">
         <v>14</v>
@@ -9198,9 +9213,6 @@
       </c>
       <c r="U116" t="s">
         <v>243</v>
-      </c>
-      <c r="W116" t="s">
-        <v>258</v>
       </c>
       <c r="AA116">
         <v>0</v>
@@ -9232,13 +9244,13 @@
         <v>147</v>
       </c>
       <c r="G117">
-        <v>9588</v>
+        <v>9600</v>
       </c>
       <c r="H117">
         <v>0</v>
       </c>
       <c r="I117" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J117" t="s">
         <v>169</v>
@@ -9246,11 +9258,14 @@
       <c r="L117" s="1">
         <v>46281</v>
       </c>
+      <c r="M117" t="s">
+        <v>212</v>
+      </c>
       <c r="N117" t="s">
         <v>221</v>
       </c>
       <c r="O117">
-        <v>17260697</v>
+        <v>17260707</v>
       </c>
       <c r="P117" t="s">
         <v>224</v>
@@ -9259,7 +9274,7 @@
         <v>237</v>
       </c>
       <c r="R117" s="1">
-        <v>46281.61917288195</v>
+        <v>46286.74416644676</v>
       </c>
       <c r="S117">
         <v>14</v>
@@ -9270,6 +9285,9 @@
       <c r="U117" t="s">
         <v>243</v>
       </c>
+      <c r="W117" t="s">
+        <v>258</v>
+      </c>
       <c r="AA117">
         <v>0</v>
       </c>
@@ -9282,16 +9300,16 @@
     </row>
     <row r="118" spans="1:33">
       <c r="A118">
-        <v>4535</v>
+        <v>4815</v>
       </c>
       <c r="B118" t="s">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="C118" t="s">
         <v>141</v>
       </c>
       <c r="D118" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E118" t="s">
         <v>147</v>
@@ -9300,13 +9318,13 @@
         <v>147</v>
       </c>
       <c r="G118">
-        <v>9600</v>
+        <v>9588</v>
       </c>
       <c r="H118">
         <v>0</v>
       </c>
       <c r="I118" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J118" t="s">
         <v>169</v>
@@ -9314,14 +9332,11 @@
       <c r="L118" s="1">
         <v>46281</v>
       </c>
-      <c r="M118" t="s">
-        <v>212</v>
-      </c>
       <c r="N118" t="s">
         <v>221</v>
       </c>
       <c r="O118">
-        <v>17260707</v>
+        <v>17728410</v>
       </c>
       <c r="P118" t="s">
         <v>224</v>
@@ -9330,7 +9345,7 @@
         <v>237</v>
       </c>
       <c r="R118" s="1">
-        <v>46286.74416644676</v>
+        <v>46281.61917341435</v>
       </c>
       <c r="S118">
         <v>14</v>
@@ -9340,9 +9355,6 @@
       </c>
       <c r="U118" t="s">
         <v>243</v>
-      </c>
-      <c r="W118" t="s">
-        <v>258</v>
       </c>
       <c r="AA118">
         <v>0</v>
@@ -9374,13 +9386,13 @@
         <v>147</v>
       </c>
       <c r="G119">
-        <v>9588</v>
+        <v>9600</v>
       </c>
       <c r="H119">
         <v>0</v>
       </c>
       <c r="I119" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J119" t="s">
         <v>169</v>
@@ -9388,11 +9400,14 @@
       <c r="L119" s="1">
         <v>46281</v>
       </c>
+      <c r="M119" t="s">
+        <v>212</v>
+      </c>
       <c r="N119" t="s">
         <v>221</v>
       </c>
       <c r="O119">
-        <v>17728410</v>
+        <v>17728420</v>
       </c>
       <c r="P119" t="s">
         <v>224</v>
@@ -9401,7 +9416,7 @@
         <v>237</v>
       </c>
       <c r="R119" s="1">
-        <v>46281.61917341435</v>
+        <v>46286.74416686343</v>
       </c>
       <c r="S119">
         <v>14</v>
@@ -9412,6 +9427,9 @@
       <c r="U119" t="s">
         <v>243</v>
       </c>
+      <c r="W119" t="s">
+        <v>258</v>
+      </c>
       <c r="AA119">
         <v>0</v>
       </c>
@@ -9424,16 +9442,16 @@
     </row>
     <row r="120" spans="1:33">
       <c r="A120">
-        <v>4815</v>
+        <v>4059</v>
       </c>
       <c r="B120" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="C120" t="s">
         <v>141</v>
       </c>
       <c r="D120" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E120" t="s">
         <v>147</v>
@@ -9442,28 +9460,25 @@
         <v>147</v>
       </c>
       <c r="G120">
-        <v>9600</v>
+        <v>11293</v>
       </c>
       <c r="H120">
         <v>0</v>
       </c>
       <c r="I120" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J120" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="L120" s="1">
-        <v>46281</v>
-      </c>
-      <c r="M120" t="s">
-        <v>212</v>
+        <v>46267</v>
       </c>
       <c r="N120" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O120">
-        <v>17728420</v>
+        <v>17311936</v>
       </c>
       <c r="P120" t="s">
         <v>224</v>
@@ -9472,10 +9487,10 @@
         <v>237</v>
       </c>
       <c r="R120" s="1">
-        <v>46286.74416686343</v>
+        <v>46267.65902924768</v>
       </c>
       <c r="S120">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="T120" t="s">
         <v>238</v>
@@ -9483,9 +9498,6 @@
       <c r="U120" t="s">
         <v>243</v>
       </c>
-      <c r="W120" t="s">
-        <v>258</v>
-      </c>
       <c r="AA120">
         <v>0</v>
       </c>
@@ -9498,10 +9510,10 @@
     </row>
     <row r="121" spans="1:33">
       <c r="A121">
-        <v>4059</v>
+        <v>4061</v>
       </c>
       <c r="B121" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C121" t="s">
         <v>141</v>
@@ -9510,7 +9522,7 @@
         <v>144</v>
       </c>
       <c r="E121" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F121" t="s">
         <v>147</v>
@@ -9522,7 +9534,7 @@
         <v>0</v>
       </c>
       <c r="I121" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J121" t="s">
         <v>178</v>
@@ -9534,7 +9546,7 @@
         <v>220</v>
       </c>
       <c r="O121">
-        <v>17311936</v>
+        <v>17311986</v>
       </c>
       <c r="P121" t="s">
         <v>224</v>
@@ -9543,7 +9555,7 @@
         <v>237</v>
       </c>
       <c r="R121" s="1">
-        <v>46267.65902924768</v>
+        <v>46267.65903065972</v>
       </c>
       <c r="S121">
         <v>28</v>
@@ -9566,10 +9578,10 @@
     </row>
     <row r="122" spans="1:33">
       <c r="A122">
-        <v>4061</v>
+        <v>4062</v>
       </c>
       <c r="B122" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C122" t="s">
         <v>141</v>
@@ -9578,7 +9590,7 @@
         <v>144</v>
       </c>
       <c r="E122" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F122" t="s">
         <v>147</v>
@@ -9590,7 +9602,7 @@
         <v>0</v>
       </c>
       <c r="I122" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J122" t="s">
         <v>178</v>
@@ -9602,7 +9614,7 @@
         <v>220</v>
       </c>
       <c r="O122">
-        <v>17311986</v>
+        <v>17756726</v>
       </c>
       <c r="P122" t="s">
         <v>224</v>
@@ -9611,7 +9623,7 @@
         <v>237</v>
       </c>
       <c r="R122" s="1">
-        <v>46267.65903065972</v>
+        <v>46267.65903172454</v>
       </c>
       <c r="S122">
         <v>28</v>
@@ -9634,10 +9646,10 @@
     </row>
     <row r="123" spans="1:33">
       <c r="A123">
-        <v>4062</v>
+        <v>4063</v>
       </c>
       <c r="B123" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C123" t="s">
         <v>141</v>
@@ -9646,7 +9658,7 @@
         <v>144</v>
       </c>
       <c r="E123" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F123" t="s">
         <v>147</v>
@@ -9658,7 +9670,7 @@
         <v>0</v>
       </c>
       <c r="I123" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J123" t="s">
         <v>178</v>
@@ -9670,7 +9682,7 @@
         <v>220</v>
       </c>
       <c r="O123">
-        <v>17756726</v>
+        <v>17221940</v>
       </c>
       <c r="P123" t="s">
         <v>224</v>
@@ -9679,7 +9691,7 @@
         <v>237</v>
       </c>
       <c r="R123" s="1">
-        <v>46267.65903172454</v>
+        <v>46267.65903244213</v>
       </c>
       <c r="S123">
         <v>28</v>
@@ -9702,10 +9714,10 @@
     </row>
     <row r="124" spans="1:33">
       <c r="A124">
-        <v>4063</v>
+        <v>4535</v>
       </c>
       <c r="B124" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C124" t="s">
         <v>141</v>
@@ -9714,7 +9726,7 @@
         <v>144</v>
       </c>
       <c r="E124" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F124" t="s">
         <v>147</v>
@@ -9726,7 +9738,7 @@
         <v>0</v>
       </c>
       <c r="I124" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J124" t="s">
         <v>178</v>
@@ -9738,7 +9750,7 @@
         <v>220</v>
       </c>
       <c r="O124">
-        <v>17221940</v>
+        <v>17260716</v>
       </c>
       <c r="P124" t="s">
         <v>224</v>
@@ -9747,7 +9759,7 @@
         <v>237</v>
       </c>
       <c r="R124" s="1">
-        <v>46267.65903244213</v>
+        <v>46267.65903319445</v>
       </c>
       <c r="S124">
         <v>28</v>
@@ -9770,16 +9782,16 @@
     </row>
     <row r="125" spans="1:33">
       <c r="A125">
-        <v>4535</v>
+        <v>4815</v>
       </c>
       <c r="B125" t="s">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="C125" t="s">
         <v>141</v>
       </c>
       <c r="D125" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E125" t="s">
         <v>147</v>
@@ -9794,7 +9806,7 @@
         <v>0</v>
       </c>
       <c r="I125" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J125" t="s">
         <v>178</v>
@@ -9806,7 +9818,7 @@
         <v>220</v>
       </c>
       <c r="O125">
-        <v>17260716</v>
+        <v>17728429</v>
       </c>
       <c r="P125" t="s">
         <v>224</v>
@@ -9815,7 +9827,7 @@
         <v>237</v>
       </c>
       <c r="R125" s="1">
-        <v>46267.65903319445</v>
+        <v>46267.65903408565</v>
       </c>
       <c r="S125">
         <v>28</v>
@@ -9838,16 +9850,16 @@
     </row>
     <row r="126" spans="1:33">
       <c r="A126">
-        <v>4815</v>
+        <v>4059</v>
       </c>
       <c r="B126" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="C126" t="s">
         <v>141</v>
       </c>
       <c r="D126" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E126" t="s">
         <v>147</v>
@@ -9856,25 +9868,25 @@
         <v>147</v>
       </c>
       <c r="G126">
-        <v>11293</v>
+        <v>9570</v>
       </c>
       <c r="H126">
         <v>0</v>
       </c>
       <c r="I126" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J126" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L126" s="1">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="N126" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O126">
-        <v>17728429</v>
+        <v>17311907</v>
       </c>
       <c r="P126" t="s">
         <v>224</v>
@@ -9883,10 +9895,10 @@
         <v>237</v>
       </c>
       <c r="R126" s="1">
-        <v>46267.65903408565</v>
+        <v>46266.65725641204</v>
       </c>
       <c r="S126">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T126" t="s">
         <v>238</v>
@@ -9901,15 +9913,15 @@
         <v>224</v>
       </c>
       <c r="AG126" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="127" spans="1:33">
       <c r="A127">
-        <v>4059</v>
+        <v>4061</v>
       </c>
       <c r="B127" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C127" t="s">
         <v>141</v>
@@ -9918,7 +9930,7 @@
         <v>144</v>
       </c>
       <c r="E127" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F127" t="s">
         <v>147</v>
@@ -9930,7 +9942,7 @@
         <v>0</v>
       </c>
       <c r="I127" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J127" t="s">
         <v>179</v>
@@ -9942,7 +9954,7 @@
         <v>221</v>
       </c>
       <c r="O127">
-        <v>17311907</v>
+        <v>17311957</v>
       </c>
       <c r="P127" t="s">
         <v>224</v>
@@ -9951,7 +9963,7 @@
         <v>237</v>
       </c>
       <c r="R127" s="1">
-        <v>46266.65725641204</v>
+        <v>46266.65725738426</v>
       </c>
       <c r="S127">
         <v>29</v>
@@ -9974,10 +9986,10 @@
     </row>
     <row r="128" spans="1:33">
       <c r="A128">
-        <v>4061</v>
+        <v>4062</v>
       </c>
       <c r="B128" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C128" t="s">
         <v>141</v>
@@ -9986,7 +9998,7 @@
         <v>144</v>
       </c>
       <c r="E128" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F128" t="s">
         <v>147</v>
@@ -9998,7 +10010,7 @@
         <v>0</v>
       </c>
       <c r="I128" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J128" t="s">
         <v>179</v>
@@ -10010,7 +10022,7 @@
         <v>221</v>
       </c>
       <c r="O128">
-        <v>17311957</v>
+        <v>17756697</v>
       </c>
       <c r="P128" t="s">
         <v>224</v>
@@ -10019,7 +10031,7 @@
         <v>237</v>
       </c>
       <c r="R128" s="1">
-        <v>46266.65725738426</v>
+        <v>46266.65725806713</v>
       </c>
       <c r="S128">
         <v>29</v>
@@ -10042,10 +10054,10 @@
     </row>
     <row r="129" spans="1:33">
       <c r="A129">
-        <v>4062</v>
+        <v>4063</v>
       </c>
       <c r="B129" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C129" t="s">
         <v>141</v>
@@ -10054,7 +10066,7 @@
         <v>144</v>
       </c>
       <c r="E129" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F129" t="s">
         <v>147</v>
@@ -10066,7 +10078,7 @@
         <v>0</v>
       </c>
       <c r="I129" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J129" t="s">
         <v>179</v>
@@ -10078,7 +10090,7 @@
         <v>221</v>
       </c>
       <c r="O129">
-        <v>17756697</v>
+        <v>17221863</v>
       </c>
       <c r="P129" t="s">
         <v>224</v>
@@ -10087,7 +10099,7 @@
         <v>237</v>
       </c>
       <c r="R129" s="1">
-        <v>46266.65725806713</v>
+        <v>46266.65725861111</v>
       </c>
       <c r="S129">
         <v>29</v>
@@ -10110,10 +10122,10 @@
     </row>
     <row r="130" spans="1:33">
       <c r="A130">
-        <v>4063</v>
+        <v>4535</v>
       </c>
       <c r="B130" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C130" t="s">
         <v>141</v>
@@ -10122,7 +10134,7 @@
         <v>144</v>
       </c>
       <c r="E130" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F130" t="s">
         <v>147</v>
@@ -10134,7 +10146,7 @@
         <v>0</v>
       </c>
       <c r="I130" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J130" t="s">
         <v>179</v>
@@ -10146,7 +10158,7 @@
         <v>221</v>
       </c>
       <c r="O130">
-        <v>17221863</v>
+        <v>17260687</v>
       </c>
       <c r="P130" t="s">
         <v>224</v>
@@ -10155,7 +10167,7 @@
         <v>237</v>
       </c>
       <c r="R130" s="1">
-        <v>46266.65725861111</v>
+        <v>46266.65725960648</v>
       </c>
       <c r="S130">
         <v>29</v>
@@ -10178,16 +10190,16 @@
     </row>
     <row r="131" spans="1:33">
       <c r="A131">
-        <v>4535</v>
+        <v>4917</v>
       </c>
       <c r="B131" t="s">
-        <v>86</v>
+        <v>36</v>
       </c>
       <c r="C131" t="s">
         <v>141</v>
       </c>
       <c r="D131" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E131" t="s">
         <v>147</v>
@@ -10196,25 +10208,28 @@
         <v>147</v>
       </c>
       <c r="G131">
-        <v>9570</v>
+        <v>9277</v>
       </c>
       <c r="H131">
         <v>0</v>
       </c>
       <c r="I131" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="J131" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="L131" s="1">
-        <v>46266</v>
+        <v>46295</v>
+      </c>
+      <c r="M131" t="s">
+        <v>211</v>
       </c>
       <c r="N131" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="O131">
-        <v>17260687</v>
+        <v>17629821</v>
       </c>
       <c r="P131" t="s">
         <v>224</v>
@@ -10223,16 +10238,19 @@
         <v>237</v>
       </c>
       <c r="R131" s="1">
-        <v>46266.65725960648</v>
+        <v>46295.40261266204</v>
       </c>
       <c r="S131">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="T131" t="s">
         <v>238</v>
       </c>
       <c r="U131" t="s">
         <v>243</v>
+      </c>
+      <c r="W131" t="s">
+        <v>254</v>
       </c>
       <c r="AA131">
         <v>0</v>
@@ -55060,7 +55078,7 @@
         <v>2143</v>
       </c>
       <c r="I765" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J765" t="s">
         <v>201</v>
@@ -55134,7 +55152,7 @@
         <v>2143</v>
       </c>
       <c r="I766" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J766" t="s">
         <v>201</v>
@@ -55208,7 +55226,7 @@
         <v>2143</v>
       </c>
       <c r="I767" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J767" t="s">
         <v>202</v>
@@ -55282,7 +55300,7 @@
         <v>2143</v>
       </c>
       <c r="I768" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J768" t="s">
         <v>203</v>
@@ -55356,7 +55374,7 @@
         <v>2143</v>
       </c>
       <c r="I769" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J769" t="s">
         <v>204</v>
@@ -55430,7 +55448,7 @@
         <v>2143</v>
       </c>
       <c r="I770" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J770" t="s">
         <v>205</v>
@@ -55504,7 +55522,7 @@
         <v>2143</v>
       </c>
       <c r="I771" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J771" t="s">
         <v>205</v>
@@ -55578,7 +55596,7 @@
         <v>2143</v>
       </c>
       <c r="I772" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J772" t="s">
         <v>206</v>
@@ -55652,7 +55670,7 @@
         <v>2143</v>
       </c>
       <c r="I773" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J773" t="s">
         <v>190</v>
@@ -55726,7 +55744,7 @@
         <v>2143</v>
       </c>
       <c r="I774" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J774" t="s">
         <v>190</v>
@@ -55800,7 +55818,7 @@
         <v>0</v>
       </c>
       <c r="I775" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J775" t="s">
         <v>172</v>
@@ -55874,7 +55892,7 @@
         <v>0</v>
       </c>
       <c r="I776" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J776" t="s">
         <v>172</v>
@@ -55948,7 +55966,7 @@
         <v>0</v>
       </c>
       <c r="I777" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J777" t="s">
         <v>207</v>
@@ -56022,7 +56040,7 @@
         <v>0</v>
       </c>
       <c r="I778" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J778" t="s">
         <v>207</v>
@@ -56096,7 +56114,7 @@
         <v>0</v>
       </c>
       <c r="I779" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J779" t="s">
         <v>167</v>
@@ -56170,7 +56188,7 @@
         <v>0</v>
       </c>
       <c r="I780" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J780" t="s">
         <v>167</v>
@@ -56244,7 +56262,7 @@
         <v>0</v>
       </c>
       <c r="I781" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J781" t="s">
         <v>170</v>
@@ -56315,7 +56333,7 @@
         <v>0</v>
       </c>
       <c r="I782" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J782" t="s">
         <v>181</v>
@@ -56389,7 +56407,7 @@
         <v>0</v>
       </c>
       <c r="I783" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J783" t="s">
         <v>181</v>
@@ -56463,7 +56481,7 @@
         <v>0</v>
       </c>
       <c r="I784" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J784" t="s">
         <v>199</v>
@@ -56531,7 +56549,7 @@
         <v>0</v>
       </c>
       <c r="I785" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J785" t="s">
         <v>199</v>
@@ -56599,7 +56617,7 @@
         <v>0</v>
       </c>
       <c r="I786" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J786" t="s">
         <v>199</v>
@@ -56667,7 +56685,7 @@
         <v>0</v>
       </c>
       <c r="I787" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J787" t="s">
         <v>199</v>
@@ -56735,7 +56753,7 @@
         <v>0</v>
       </c>
       <c r="I788" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J788" t="s">
         <v>199</v>
@@ -56803,7 +56821,7 @@
         <v>0</v>
       </c>
       <c r="I789" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J789" t="s">
         <v>199</v>
@@ -56871,7 +56889,7 @@
         <v>0</v>
       </c>
       <c r="I790" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J790" t="s">
         <v>188</v>
@@ -56939,7 +56957,7 @@
         <v>0</v>
       </c>
       <c r="I791" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J791" t="s">
         <v>188</v>
@@ -57007,7 +57025,7 @@
         <v>0</v>
       </c>
       <c r="I792" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J792" t="s">
         <v>188</v>
@@ -57075,7 +57093,7 @@
         <v>0</v>
       </c>
       <c r="I793" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J793" t="s">
         <v>188</v>
@@ -57143,7 +57161,7 @@
         <v>0</v>
       </c>
       <c r="I794" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J794" t="s">
         <v>188</v>
@@ -57211,7 +57229,7 @@
         <v>0</v>
       </c>
       <c r="I795" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J795" t="s">
         <v>188</v>
@@ -57279,7 +57297,7 @@
         <v>0</v>
       </c>
       <c r="I796" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J796" t="s">
         <v>188</v>
@@ -57347,7 +57365,7 @@
         <v>0</v>
       </c>
       <c r="I797" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J797" t="s">
         <v>188</v>
@@ -57415,7 +57433,7 @@
         <v>0</v>
       </c>
       <c r="I798" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J798" t="s">
         <v>188</v>
@@ -57483,7 +57501,7 @@
         <v>0</v>
       </c>
       <c r="I799" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J799" t="s">
         <v>188</v>
@@ -57551,7 +57569,7 @@
         <v>0</v>
       </c>
       <c r="I800" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J800" t="s">
         <v>188</v>
@@ -57619,7 +57637,7 @@
         <v>0</v>
       </c>
       <c r="I801" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J801" t="s">
         <v>188</v>
@@ -57687,7 +57705,7 @@
         <v>0</v>
       </c>
       <c r="I802" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J802" t="s">
         <v>188</v>
@@ -57755,7 +57773,7 @@
         <v>0</v>
       </c>
       <c r="I803" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J803" t="s">
         <v>188</v>
@@ -57823,7 +57841,7 @@
         <v>0</v>
       </c>
       <c r="I804" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J804" t="s">
         <v>188</v>
@@ -57891,7 +57909,7 @@
         <v>2143</v>
       </c>
       <c r="I805" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J805" t="s">
         <v>200</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-29 12:43
</commit_message>
<xml_diff>
--- a/dados/base/bpo.xlsx
+++ b/dados/base/bpo.xlsx
@@ -5322,7 +5322,7 @@
         <v>142</v>
       </c>
       <c r="E64" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F64" t="s">
         <v>147</v>
@@ -5446,7 +5446,7 @@
         <v>142</v>
       </c>
       <c r="E66" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F66" t="s">
         <v>147</v>
@@ -10902,7 +10902,7 @@
         <v>142</v>
       </c>
       <c r="E154" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F154" t="s">
         <v>147</v>
@@ -15724,7 +15724,7 @@
         <v>142</v>
       </c>
       <c r="E222" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F222" t="s">
         <v>147</v>
@@ -15872,7 +15872,7 @@
         <v>142</v>
       </c>
       <c r="E224" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F224" t="s">
         <v>147</v>
@@ -16020,7 +16020,7 @@
         <v>142</v>
       </c>
       <c r="E226" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F226" t="s">
         <v>147</v>
@@ -56567,7 +56567,7 @@
         <v>142</v>
       </c>
       <c r="E806" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F806" t="s">
         <v>147</v>
@@ -56703,7 +56703,7 @@
         <v>142</v>
       </c>
       <c r="E808" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F808" t="s">
         <v>147</v>
@@ -56771,7 +56771,7 @@
         <v>142</v>
       </c>
       <c r="E809" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F809" t="s">
         <v>147</v>
@@ -56839,7 +56839,7 @@
         <v>142</v>
       </c>
       <c r="E810" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F810" t="s">
         <v>147</v>
@@ -56907,7 +56907,7 @@
         <v>142</v>
       </c>
       <c r="E811" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F811" t="s">
         <v>147</v>
@@ -57043,7 +57043,7 @@
         <v>142</v>
       </c>
       <c r="E813" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F813" t="s">
         <v>147</v>
@@ -57111,7 +57111,7 @@
         <v>142</v>
       </c>
       <c r="E814" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F814" t="s">
         <v>147</v>
@@ -57247,7 +57247,7 @@
         <v>142</v>
       </c>
       <c r="E816" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F816" t="s">
         <v>147</v>
@@ -57383,7 +57383,7 @@
         <v>142</v>
       </c>
       <c r="E818" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F818" t="s">
         <v>147</v>
@@ -57531,7 +57531,7 @@
         <v>142</v>
       </c>
       <c r="E820" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F820" t="s">
         <v>147</v>
@@ -57679,7 +57679,7 @@
         <v>142</v>
       </c>
       <c r="E822" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F822" t="s">
         <v>147</v>
@@ -57753,7 +57753,7 @@
         <v>142</v>
       </c>
       <c r="E823" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F823" t="s">
         <v>147</v>
@@ -57969,7 +57969,7 @@
         <v>142</v>
       </c>
       <c r="E826" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F826" t="s">
         <v>147</v>
@@ -58117,7 +58117,7 @@
         <v>142</v>
       </c>
       <c r="E828" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F828" t="s">
         <v>147</v>
@@ -58525,7 +58525,7 @@
         <v>142</v>
       </c>
       <c r="E834" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F834" t="s">
         <v>147</v>
@@ -59551,7 +59551,7 @@
         <v>142</v>
       </c>
       <c r="E849" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F849" t="s">
         <v>147</v>
@@ -59687,7 +59687,7 @@
         <v>142</v>
       </c>
       <c r="E851" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F851" t="s">
         <v>147</v>
@@ -59755,7 +59755,7 @@
         <v>142</v>
       </c>
       <c r="E852" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F852" t="s">
         <v>147</v>
@@ -60347,7 +60347,7 @@
         <v>142</v>
       </c>
       <c r="E860" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F860" t="s">
         <v>147</v>

</xml_diff>